<commit_message>
Republish Tesla (TSLA) study — corrected five-lens synthesis (weighted central USD 254, −40%; autonomy-at-scale carries 25% weight) and rebuilt three-expert panel (Expert 3 scenario real-options ~USD 350, near spot); refresh docx/pdf/xlsx, data.js fair {105/254/350}, EN+AR pages and listings; file token v=0108, site cache-bust v=20260701f
</commit_message>
<xml_diff>
--- a/files/TSLA_Valuation_Model_30-06-2026_public.xlsx
+++ b/files/TSLA_Valuation_Model_30-06-2026_public.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="302">
   <si>
     <t xml:space="preserve">Testahil — Independent Valuation Study — Educational Analysis</t>
   </si>
@@ -85,10 +85,10 @@
     <t xml:space="preserve">Valuation range (USD/sh)</t>
   </si>
   <si>
-    <t xml:space="preserve">SOTP — base (primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DCF — cross-check</t>
+    <t xml:space="preserve">SOTP — segments + option (primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCF — cross-check (floor)</t>
   </si>
   <si>
     <t xml:space="preserve">Relative (blended)</t>
@@ -97,7 +97,7 @@
     <t xml:space="preserve">Normalized earnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Autonomy-at-scale (SOTP bull)</t>
+    <t xml:space="preserve">Autonomy-at-scale (SOTP bull, ceiling)</t>
   </si>
   <si>
     <t xml:space="preserve">Monte Carlo (3-month, 50k paths, seed 42)</t>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">Read: richly valued on fundamentals; the case is an autonomy/AI optionality bet. This is a valuation, not advice.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fundamental valuation — four lenses</t>
+    <t xml:space="preserve">Fundamental valuation — five lenses</t>
   </si>
   <si>
     <t xml:space="preserve">DCF is the primary anchor; SOTP isolates the autonomy option. All values link from their sheets.</t>
@@ -127,10 +127,7 @@
     <t xml:space="preserve">Weight</t>
   </si>
   <si>
-    <t xml:space="preserve">SOTP — segments + option (primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consolidated DCF (cross-check)</t>
+    <t xml:space="preserve">Consolidated DCF (cross-check) — floor</t>
   </si>
   <si>
     <t xml:space="preserve">Relative multiples (blended)</t>
@@ -139,19 +136,19 @@
     <t xml:space="preserve">Normalized earnings power</t>
   </si>
   <si>
+    <t xml:space="preserve">Autonomy-at-scale (SOTP bull) — ceiling</t>
+  </si>
+  <si>
     <t xml:space="preserve">WEIGHTED CENTRAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Memo: autonomy-at-scale (SOTP bull)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Memo: spot (USD)</t>
   </si>
   <si>
     <t xml:space="preserve">Memo: Monte Carlo T+60 median (USD)</t>
   </si>
   <si>
-    <t xml:space="preserve">All four operating lenses sit below spot; only the autonomy-at-scale case exceeds it. The dispersion is the widest in coverage.</t>
+    <t xml:space="preserve">Four of the five lenses sit below spot; only the autonomy-at-scale case exceeds it, and it carries a full quarter of the weight. The dispersion (USD 90–560) is the widest in coverage and is driven almost entirely by the value of the autonomy option.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions — single input layer</t>
@@ -262,16 +259,13 @@
     <t xml:space="preserve">Normalized earnings — power lens (USD bn)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lens weights (synthesis — four lenses)</t>
+    <t xml:space="preserve">Lens weights (synthesis — five lenses)</t>
   </si>
   <si>
     <t xml:space="preserve">Relative multiples</t>
   </si>
   <si>
     <t xml:space="preserve">Weights total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memo: autonomy-at-scale (SOTP bull, not weighted)</t>
   </si>
   <si>
     <t xml:space="preserve">Segment sum-of-the-parts — isolating the optionality</t>
@@ -1623,46 +1617,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="G4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="H4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="I4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>16.4</v>
@@ -1691,7 +1685,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>12.7</v>
@@ -1720,7 +1714,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>3.5</v>
@@ -1749,7 +1743,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>13.6</v>
@@ -1778,7 +1772,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B9" s="31" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -1815,7 +1809,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B10" s="21" t="n">
         <v>29.7</v>
@@ -1844,7 +1838,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B11" s="21" t="n">
         <v>30.9</v>
@@ -1873,7 +1867,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B12" s="31" t="n">
         <f aca="false">B9+B10+B11</f>
@@ -1910,7 +1904,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B13" s="21" t="n">
         <v>23.8</v>
@@ -1939,7 +1933,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B14" s="21" t="n">
         <v>9.6</v>
@@ -1968,7 +1962,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B15" s="21" t="n">
         <v>10.5</v>
@@ -1997,7 +1991,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B16" s="31" t="n">
         <f aca="false">B13+B14+B15</f>
@@ -2034,7 +2028,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B17" s="31" t="n">
         <f aca="false">B12-B16</f>
@@ -2071,7 +2065,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B5+B6-B14</f>
@@ -2108,7 +2102,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2136,46 +2130,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="G4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="H4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="I4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>13.3</v>
@@ -2204,7 +2198,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>-8.9</v>
@@ -2238,7 +2232,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B7" s="31" t="n">
         <f aca="false">B5+B6</f>
@@ -2275,7 +2269,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2303,46 +2297,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="G4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="H4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="I4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B5" s="30" t="n">
         <f aca="false">'Income Statement'!B8</f>
@@ -2379,7 +2373,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">'Income Statement'!B12</f>
@@ -2416,7 +2410,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">'Income Statement'!B12/'Income Statement'!B8</f>
@@ -2453,7 +2447,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B8" s="30" t="n">
         <f aca="false">'Income Statement'!B16</f>
@@ -2490,7 +2484,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">'Income Statement'!B17</f>
@@ -2527,7 +2521,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">'Balance Sheet'!B12</f>
@@ -2564,7 +2558,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">'Balance Sheet'!B17</f>
@@ -2601,7 +2595,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B12" s="30" t="n">
         <f aca="false">'Balance Sheet'!B18</f>
@@ -2638,7 +2632,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B13" s="30" t="n">
         <f aca="false">'Cash Flow'!B5</f>
@@ -2675,7 +2669,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B14" s="30" t="n">
         <f aca="false">'Cash Flow'!B7</f>
@@ -2735,22 +2729,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B5" s="7" t="n">
         <f aca="false">Assumptions!B5</f>
@@ -2759,7 +2753,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B6" s="22" t="n">
         <v>0.48</v>
@@ -2767,7 +2761,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>0.029</v>
@@ -2775,7 +2769,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>0.554</v>
@@ -2783,32 +2777,32 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="C11" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="D11" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="E11" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="F11" s="15" t="s">
         <v>205</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>206</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B12" s="28" t="n">
         <v>325</v>
@@ -2828,7 +2822,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B13" s="28" t="n">
         <v>270</v>
@@ -2848,21 +2842,21 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>210</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="D16" s="15" t="s">
         <v>212</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2876,7 +2870,7 @@
         <v>0.68</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2890,7 +2884,7 @@
         <v>0.54</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2904,7 +2898,7 @@
         <v>0.46</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E19" s="28" t="n">
         <v>501</v>
@@ -2924,7 +2918,7 @@
         <v>0.3</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2938,7 +2932,7 @@
         <v>0.65</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2952,7 +2946,7 @@
         <v>0.51</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2966,7 +2960,7 @@
         <v>0.28</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,132 +2974,132 @@
         <v>0.15</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="D27" s="15" t="s">
         <v>225</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C28" s="22" t="n">
         <v>-0.005</v>
       </c>
       <c r="D28" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C29" s="22" t="n">
         <v>0.01</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B30" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C30" s="22" t="n">
         <v>0.01</v>
       </c>
       <c r="D30" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C31" s="22" t="n">
         <v>-0.006</v>
       </c>
       <c r="D31" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B32" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C32" s="22" t="n">
         <v>0.014</v>
       </c>
       <c r="D32" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B33" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C33" s="22" t="n">
         <v>0.006</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B34" s="39" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C34" s="22" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="39" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C35" s="22" t="n">
         <v>0.08</v>
@@ -3116,10 +3110,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C36" s="22" t="n">
         <v>0.01</v>
@@ -3130,10 +3124,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C37" s="22" t="n">
         <v>0</v>
@@ -3144,10 +3138,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C38" s="22" t="n">
         <v>0.06</v>
@@ -3158,10 +3152,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C39" s="22" t="n">
         <v>-0.07</v>
@@ -3172,10 +3166,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B40" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C40" s="22" t="n">
         <v>-0.06</v>
@@ -3186,10 +3180,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C41" s="22" t="n">
         <v>-0.01</v>
@@ -3200,10 +3194,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C42" s="22" t="n">
         <v>-0.06</v>
@@ -3214,10 +3208,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C43" s="22" t="n">
         <v>0.04</v>
@@ -3228,7 +3222,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3256,17 +3250,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B4" s="41" t="n">
         <v>0.03</v>
@@ -3411,7 +3405,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -3439,17 +3433,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B4" s="7" t="n">
         <f aca="false">Assumptions!B5</f>
@@ -3476,7 +3470,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B7" s="30" t="n">
         <f aca="false">Assumptions!B7</f>
@@ -3485,7 +3479,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B6-B7</f>
@@ -3494,12 +3488,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">'Income Statement'!D17</f>
@@ -3508,7 +3502,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B12" s="43" t="n">
         <f aca="false">B4/B11</f>
@@ -3517,7 +3511,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13" s="30" t="n">
         <f aca="false">'Income Statement'!D8</f>
@@ -3526,7 +3520,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B14" s="43" t="n">
         <f aca="false">B8/B13</f>
@@ -3535,12 +3529,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B17" s="7" t="n">
         <f aca="false">'Income Statement'!F17</f>
@@ -3549,7 +3543,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B18" s="43" t="n">
         <f aca="false">B4/B17</f>
@@ -3558,7 +3552,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B19" s="30" t="n">
         <f aca="false">'Income Statement'!F8</f>
@@ -3567,7 +3561,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B20" s="43" t="n">
         <f aca="false">B8/B19</f>
@@ -3576,30 +3570,30 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B23" s="11" t="n">
-        <f aca="false">'Fundamental Valuation'!B9</f>
-        <v>174.120289751186</v>
+        <f aca="false">'Fundamental Valuation'!B10</f>
+        <v>254.009037111583</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B24" s="43" t="n">
         <f aca="false">B23/B17</f>
-        <v>49.7486542146246</v>
+        <v>72.5740106033095</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3628,145 +3622,145 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>270</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>271</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>272</v>
-      </c>
       <c r="D4" s="15" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" s="44" t="s">
         <v>273</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="C5" s="44" t="s">
-        <v>275</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="C6" s="44" t="s">
         <v>277</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>278</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>279</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="C7" s="44" t="s">
         <v>281</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="C7" s="44" t="s">
-        <v>283</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="C8" s="44" t="s">
         <v>285</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>286</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>287</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="C9" s="44" t="s">
         <v>289</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>290</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>291</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C10" s="44" t="s">
         <v>293</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>294</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>295</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="45" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="45" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="45" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="45" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="45" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="45" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -3834,8 +3828,8 @@
         <v>13</v>
       </c>
       <c r="B8" s="11" t="n">
-        <f aca="false">'Fundamental Valuation'!B9</f>
-        <v>174.120289751186</v>
+        <f aca="false">'Fundamental Valuation'!B10</f>
+        <v>254.009037111583</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3844,7 +3838,7 @@
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">B8/B4-1</f>
-        <v>-0.586019282569696</v>
+        <v>-0.396079322131281</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3885,7 +3879,7 @@
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">'Relative &amp; Normalized'!B13</f>
-        <v>151.702786377709</v>
+        <v>130.030959752322</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3974,7 +3968,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">SOTP!C15</f>
@@ -3986,12 +3980,12 @@
       </c>
       <c r="D5" s="17" t="n">
         <f aca="false">Assumptions!B38</f>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">DCF!B26</f>
@@ -4003,12 +3997,12 @@
       </c>
       <c r="D6" s="17" t="n">
         <f aca="false">Assumptions!B39</f>
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" s="11" t="n">
         <f aca="false">'Relative &amp; Normalized'!D8</f>
@@ -4025,50 +4019,58 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">'Relative &amp; Normalized'!B13</f>
-        <v>151.702786377709</v>
+        <v>130.030959752322</v>
       </c>
       <c r="C8" s="16" t="n">
         <f aca="false">B8/Assumptions!B5-1</f>
-        <v>-0.639318149363507</v>
+        <v>-0.690844128025863</v>
       </c>
       <c r="D8" s="17" t="n">
         <f aca="false">Assumptions!B41</f>
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="18" t="n">
-        <f aca="false">SUMPRODUCT(B5:B8,D5:D8)</f>
-        <v>174.120289751186</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <f aca="false">B9/Assumptions!B5-1</f>
-        <v>-0.586019282569696</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <f aca="false">SUM(D5:D8)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="11" t="n">
+      <c r="A9" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <f aca="false">SOTP!C16</f>
         <v>560</v>
       </c>
+      <c r="C9" s="16" t="n">
+        <f aca="false">B9/Assumptions!B5-1</f>
+        <v>0.331431288635283</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <f aca="false">Assumptions!B42</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <f aca="false">SUMPRODUCT(B5:B9,D5:D9)</f>
+        <v>254.009037111583</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <f aca="false">B10/Assumptions!B5-1</f>
+        <v>-0.396079322131281</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <f aca="false">SUM(D5:D9)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="7" t="n">
         <f aca="false">Assumptions!B5</f>
@@ -4077,7 +4079,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">'Monte Carlo'!C19</f>
@@ -4086,7 +4088,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -4105,7 +4107,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -4114,22 +4116,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="19" t="n">
         <v>420.6</v>
@@ -4137,7 +4139,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>3.23</v>
@@ -4145,7 +4147,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>40</v>
@@ -4153,32 +4155,32 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="C10" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="D10" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="E10" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="F10" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>108</v>
@@ -4198,7 +4200,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C12" s="22" t="n">
         <v>0.065</v>
@@ -4218,7 +4220,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>6.5</v>
@@ -4238,7 +4240,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C14" s="21" t="n">
         <v>25</v>
@@ -4258,7 +4260,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C15" s="21" t="n">
         <v>1</v>
@@ -4278,7 +4280,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B17" s="22" t="n">
         <v>0.15</v>
@@ -4286,7 +4288,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>0.1</v>
@@ -4294,7 +4296,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>0.045</v>
@@ -4302,12 +4304,12 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B22" s="23" t="n">
         <v>70</v>
@@ -4315,7 +4317,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B23" s="23" t="n">
         <v>35</v>
@@ -4323,7 +4325,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24" s="23" t="n">
         <v>10</v>
@@ -4331,7 +4333,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B25" s="23" t="n">
         <v>12</v>
@@ -4339,7 +4341,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B26" s="23" t="n">
         <v>433</v>
@@ -4347,7 +4349,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B27" s="22" t="n">
         <v>0.24</v>
@@ -4355,12 +4357,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B30" s="24" t="n">
         <v>5</v>
@@ -4368,7 +4370,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B31" s="24" t="n">
         <v>30</v>
@@ -4376,7 +4378,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B32" s="24" t="n">
         <v>45</v>
@@ -4384,7 +4386,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B33" s="21" t="n">
         <v>17</v>
@@ -4392,7 +4394,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B34" s="21" t="n">
         <v>12</v>
@@ -4400,7 +4402,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B35" s="24" t="n">
         <v>35</v>
@@ -4408,15 +4410,15 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" s="21" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4424,7 +4426,7 @@
         <v>16</v>
       </c>
       <c r="B38" s="22" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4432,12 +4434,12 @@
         <v>17</v>
       </c>
       <c r="B39" s="22" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B40" s="22" t="n">
         <v>0.15</v>
@@ -4448,25 +4450,24 @@
         <v>19</v>
       </c>
       <c r="B41" s="22" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B42" s="12" t="n">
-        <f aca="false">SUM(B38:B41)</f>
+        <v>20</v>
+      </c>
+      <c r="B42" s="22" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="12" t="n">
+        <f aca="false">SUM(B38:B42)</f>
         <v>1</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B44" s="11" t="n">
-        <f aca="false">SOTP!C16</f>
-        <v>560</v>
       </c>
     </row>
   </sheetData>
@@ -4495,20 +4496,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>28</v>
@@ -4516,10 +4517,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C5" s="25" t="n">
         <f aca="false">Assumptions!B22</f>
@@ -4528,10 +4529,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">Assumptions!B23</f>
@@ -4540,10 +4541,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">Assumptions!B24</f>
@@ -4552,10 +4553,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">Assumptions!B25</f>
@@ -4564,7 +4565,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C9" s="26" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -4573,10 +4574,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C11" s="11" t="n">
         <f aca="false">Assumptions!B26</f>
@@ -4585,7 +4586,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">Assumptions!B27</f>
@@ -4594,7 +4595,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C13" s="28" t="n">
         <f aca="false">C11*C12</f>
@@ -4603,7 +4604,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C15" s="29" t="n">
         <f aca="false">C9+C13</f>
@@ -4612,7 +4613,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C16" s="26" t="n">
         <f aca="false">C9+C11</f>
@@ -4621,7 +4622,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C17" s="26" t="n">
         <f aca="false">C9</f>
@@ -4630,7 +4631,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C19" s="16" t="n">
         <f aca="false">C15/Assumptions!B5-1</f>
@@ -4639,7 +4640,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C20" s="16" t="n">
         <f aca="false">C16/Assumptions!B5-1</f>
@@ -4648,7 +4649,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C21" s="16" t="n">
         <f aca="false">C17/Assumptions!B5-1</f>
@@ -4657,7 +4658,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4685,40 +4686,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="E4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="F4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="G4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B5" s="30" t="n">
         <f aca="false">'Income Statement'!C5</f>
@@ -4747,7 +4748,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">'Income Statement'!C6</f>
@@ -4776,7 +4777,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" s="30" t="n">
         <f aca="false">'Income Statement'!C7</f>
@@ -4805,7 +4806,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B8" s="31" t="n">
         <f aca="false">SUM(B5:B7)</f>
@@ -4834,12 +4835,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B11" s="16" t="n">
         <f aca="false">G5/G8</f>
@@ -4848,7 +4849,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B12" s="16" t="n">
         <f aca="false">G6/G8</f>
@@ -4857,7 +4858,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B13" s="16" t="n">
         <f aca="false">G7/G8</f>
@@ -4890,31 +4891,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="D4" s="15" t="s">
         <v>115</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B5" s="30" t="n">
         <f aca="false">Assumptions!C11</f>
@@ -4931,7 +4932,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B6" s="30" t="n">
         <f aca="false">Assumptions!B33</f>
@@ -4948,7 +4949,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B7" s="30" t="n">
         <f aca="false">Assumptions!B34</f>
@@ -4965,7 +4966,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D8" s="29" t="n">
         <f aca="false">AVERAGE(D5:D7)</f>
@@ -4974,21 +4975,21 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">Assumptions!B36</f>
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">Assumptions!B35</f>
@@ -4997,16 +4998,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B13" s="29" t="n">
         <f aca="false">B11*B12/Assumptions!B6</f>
-        <v>151.702786377709</v>
+        <v>130.030959752322</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -5034,37 +5035,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="D4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="E4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="F4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C5" s="30" t="n">
         <f aca="false">Assumptions!C11</f>
@@ -5089,7 +5090,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">Assumptions!C12</f>
@@ -5114,7 +5115,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">C5*C6</f>
@@ -5139,7 +5140,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">C7*(1-Assumptions!$B$17)</f>
@@ -5164,7 +5165,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C9" s="30" t="n">
         <f aca="false">Assumptions!C13</f>
@@ -5189,7 +5190,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C10" s="30" t="n">
         <f aca="false">-Assumptions!C14</f>
@@ -5214,7 +5215,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C11" s="30" t="n">
         <f aca="false">-Assumptions!C15</f>
@@ -5239,7 +5240,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C12" s="31" t="n">
         <f aca="false">C8+C9+C10+C11</f>
@@ -5264,7 +5265,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>1</v>
@@ -5284,7 +5285,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C14" s="34" t="n">
         <f aca="false">1/(1+Assumptions!$B$18)^C13</f>
@@ -5309,7 +5310,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">C12*C14</f>
@@ -5334,12 +5335,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">SUM(C15:G15)</f>
@@ -5348,7 +5349,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">G12*(1+Assumptions!$B$19)/(Assumptions!$B$18-Assumptions!$B$19)</f>
@@ -5357,7 +5358,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">B20*G14</f>
@@ -5366,7 +5367,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B22" s="31" t="n">
         <f aca="false">B19+B21</f>
@@ -5375,7 +5376,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B23" s="30" t="n">
         <f aca="false">Assumptions!B7</f>
@@ -5384,7 +5385,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B24" s="31" t="n">
         <f aca="false">B22+B23</f>
@@ -5402,7 +5403,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B26" s="35" t="n">
         <f aca="false">B24/B25</f>
@@ -5420,7 +5421,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -5448,46 +5449,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>151</v>
-      </c>
       <c r="D4" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="G4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="H4" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="I4" s="15" t="s">
         <v>50</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>82.4</v>
@@ -5521,7 +5522,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>6</v>
@@ -5550,7 +5551,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>8.3</v>
@@ -5579,7 +5580,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>96.8</v>
@@ -5613,7 +5614,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="36" t="n">
@@ -5647,7 +5648,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">-(B8-B12)</f>
@@ -5684,7 +5685,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>0.092</v>
@@ -5718,7 +5719,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B12" s="31" t="n">
         <f aca="false">B8*B11</f>
@@ -5755,7 +5756,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B13" s="9" t="n">
         <v>1</v>
@@ -5784,7 +5785,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">B12+B13</f>
@@ -5821,7 +5822,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B15" s="21" t="n">
         <v>5.1</v>
@@ -5855,7 +5856,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B16" s="31" t="n">
         <f aca="false">B14+B15</f>
@@ -5892,7 +5893,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B17" s="37" t="n">
         <f aca="false">B16/Assumptions!$B$6</f>
@@ -5929,7 +5930,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>